<commit_message>
📊 添加 2026-06-21 数据
</commit_message>
<xml_diff>
--- a/漳州菜篮子_零售价格日报表.xlsx
+++ b/漳州菜篮子_零售价格日报表.xlsx
@@ -16,6 +16,7 @@
     <sheet name="06-24" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="06-23" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="06-22" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="06-21" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,6 +87,60 @@
       <b val="1"/>
       <color rgb="002E7D32"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00999999"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00999999"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -160,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -215,6 +270,56 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2928,6 +3033,1548 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>漳州菜篮子 — 零售价格日报表</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>日期：2026年06月21日（星期日） | 单位：元/500g | 数据来源：漳州菜篮子网</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>分类</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>品名</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>平均价（元/500g）</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>较上日涨跌幅</t>
+        </is>
+      </c>
+      <c r="E3" s="24" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>📂 水果（9 个品种）</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>富士苹果</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>鸭梨</t>
+        </is>
+      </c>
+      <c r="C6" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>西瓜</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="34" t="inlineStr">
+        <is>
+          <t>↓ -2.44%</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>进口莲雾</t>
+        </is>
+      </c>
+      <c r="C8" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>山竹</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D9" s="34" t="inlineStr">
+        <is>
+          <t>↓ -2.27%</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>火龙果（白肉）</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>本地香蕉</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>本地菠萝</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>↑ +1.69%</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>水果</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>荔枝（乌叶）</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>📂 肉禽蛋（10 个品种）</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>猪瘦肉</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E16" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>带皮后腿肉</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="inlineStr">
+        <is>
+          <t>排骨</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="D18" s="36" t="inlineStr">
+        <is>
+          <t>↓ -0.79%</t>
+        </is>
+      </c>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>牛腱子肉</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="n">
+        <v>45</v>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>牛腩</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="D20" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>白条鸡</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="D21" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>白条鸭（菜鸭）</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D22" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E22" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>鸡场蛋</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>肉禽蛋</t>
+        </is>
+      </c>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>鸭蛋</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D24" s="35" t="inlineStr">
+        <is>
+          <t>↑ +1.56%</t>
+        </is>
+      </c>
+      <c r="E24" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>📂 水产（6 个品种）</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>水产</t>
+        </is>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>冻带鱼（250g）</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E26" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>水产</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>草鱼（1000g）</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D27" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>水产</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="inlineStr">
+        <is>
+          <t>冻黄鱼（500g）</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="n">
+        <v>26</v>
+      </c>
+      <c r="D28" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E28" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>水产</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>鳙鱼（1500g）</t>
+        </is>
+      </c>
+      <c r="C29" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="D29" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E29" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>水产</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>白鲫鱼（350g）</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="D30" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>水产</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>活虾（10cm）</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="D31" s="37" t="inlineStr">
+        <is>
+          <t>↑ +0.70%</t>
+        </is>
+      </c>
+      <c r="E31" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>📂 粮油（24 个品种）</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>黄豆</t>
+        </is>
+      </c>
+      <c r="C33" s="28" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D33" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E33" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>绿豆</t>
+        </is>
+      </c>
+      <c r="C34" s="32" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="D34" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E34" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>晚籼米（煮干饭）</t>
+        </is>
+      </c>
+      <c r="C35" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>粳米（珍珠米煮稀饭）</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>东北米（珍珠米）5公斤小包装</t>
+        </is>
+      </c>
+      <c r="C37" s="28" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="D37" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E37" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>面粉（标准粉）</t>
+        </is>
+      </c>
+      <c r="C38" s="32" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D38" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E38" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B39" s="27" t="inlineStr">
+        <is>
+          <t>菜籽油（5L/桶）金龙鱼</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="n">
+        <v>70</v>
+      </c>
+      <c r="D39" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E39" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>大豆油（5L/桶）金龙鱼</t>
+        </is>
+      </c>
+      <c r="C40" s="32" t="n">
+        <v>63.75</v>
+      </c>
+      <c r="D40" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B41" s="27" t="inlineStr">
+        <is>
+          <t>花生油（5L/桶）金龙鱼</t>
+        </is>
+      </c>
+      <c r="C41" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="D41" s="34" t="inlineStr">
+        <is>
+          <t>↓ -1.64%</t>
+        </is>
+      </c>
+      <c r="E41" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B42" s="31" t="inlineStr">
+        <is>
+          <t>第二代食用调和油（5L/桶）金龙鱼</t>
+        </is>
+      </c>
+      <c r="C42" s="32" t="n">
+        <v>65</v>
+      </c>
+      <c r="D42" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B43" s="27" t="inlineStr">
+        <is>
+          <t>鲁花花生油（5L/桶）</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="D43" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E43" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B44" s="31" t="inlineStr">
+        <is>
+          <t>金鼠香米（斤）</t>
+        </is>
+      </c>
+      <c r="C44" s="32" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E44" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B45" s="27" t="inlineStr">
+        <is>
+          <t>广洋湖香粘米（斤）</t>
+        </is>
+      </c>
+      <c r="C45" s="28" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D45" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E45" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B46" s="31" t="inlineStr">
+        <is>
+          <t>盘锦大米（斤）</t>
+        </is>
+      </c>
+      <c r="C46" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D46" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E46" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B47" s="27" t="inlineStr">
+        <is>
+          <t>洪家鸡油粘香米（5KG/包）</t>
+        </is>
+      </c>
+      <c r="C47" s="28" t="n">
+        <v>39</v>
+      </c>
+      <c r="D47" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E47" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B48" s="31" t="inlineStr">
+        <is>
+          <t>十月稻田长粒香米（5KG/包）</t>
+        </is>
+      </c>
+      <c r="C48" s="32" t="n">
+        <v>70</v>
+      </c>
+      <c r="D48" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E48" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="inlineStr">
+        <is>
+          <t>十月稻田香稻贡米（5KG/包）</t>
+        </is>
+      </c>
+      <c r="C49" s="28" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="D49" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E49" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B50" s="31" t="inlineStr">
+        <is>
+          <t>小悦米（5KG/包）</t>
+        </is>
+      </c>
+      <c r="C50" s="32" t="n">
+        <v>48</v>
+      </c>
+      <c r="D50" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E50" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B51" s="27" t="inlineStr">
+        <is>
+          <t>九三非转基因大豆油（10L/桶）</t>
+        </is>
+      </c>
+      <c r="C51" s="28" t="n">
+        <v>160</v>
+      </c>
+      <c r="D51" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E51" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B52" s="31" t="inlineStr">
+        <is>
+          <t>九三压榨浓香花生油（5L/桶）</t>
+        </is>
+      </c>
+      <c r="C52" s="32" t="n">
+        <v>158</v>
+      </c>
+      <c r="D52" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E52" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B53" s="27" t="inlineStr">
+        <is>
+          <t>馒头粉（斤）</t>
+        </is>
+      </c>
+      <c r="C53" s="28" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D53" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E53" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B54" s="31" t="inlineStr">
+        <is>
+          <t>玉米淀粉（斤）</t>
+        </is>
+      </c>
+      <c r="C54" s="32" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D54" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E54" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B55" s="27" t="inlineStr">
+        <is>
+          <t>大树碱面（1500g/件）</t>
+        </is>
+      </c>
+      <c r="C55" s="28" t="n">
+        <v>41</v>
+      </c>
+      <c r="D55" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E55" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="30" t="inlineStr">
+        <is>
+          <t>粮油</t>
+        </is>
+      </c>
+      <c r="B56" s="31" t="inlineStr">
+        <is>
+          <t>糯米</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D56" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E56" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="24" customHeight="1">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>📂 其它（7 个品种）</t>
+        </is>
+      </c>
+      <c r="B57" s="19" t="n"/>
+      <c r="C57" s="19" t="n"/>
+      <c r="D57" s="19" t="n"/>
+      <c r="E57" s="19" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="30" t="inlineStr">
+        <is>
+          <t>其它</t>
+        </is>
+      </c>
+      <c r="B58" s="31" t="inlineStr">
+        <is>
+          <t>香菇</t>
+        </is>
+      </c>
+      <c r="C58" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="D58" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E58" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="26" t="inlineStr">
+        <is>
+          <t>其它</t>
+        </is>
+      </c>
+      <c r="B59" s="27" t="inlineStr">
+        <is>
+          <t>水豆腐（块）</t>
+        </is>
+      </c>
+      <c r="C59" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E59" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="30" t="inlineStr">
+        <is>
+          <t>其它</t>
+        </is>
+      </c>
+      <c r="B60" s="31" t="inlineStr">
+        <is>
+          <t>晶华自然盐（400g/袋）</t>
+        </is>
+      </c>
+      <c r="C60" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E60" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="26" t="inlineStr">
+        <is>
+          <t>其它</t>
+        </is>
+      </c>
+      <c r="B61" s="27" t="inlineStr">
+        <is>
+          <t>冰度白砂糖（400g/袋）</t>
+        </is>
+      </c>
+      <c r="C61" s="28" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D61" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E61" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="30" t="inlineStr">
+        <is>
+          <t>其它</t>
+        </is>
+      </c>
+      <c r="B62" s="31" t="inlineStr">
+        <is>
+          <t>冰度红糖（400g/袋）</t>
+        </is>
+      </c>
+      <c r="C62" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="D62" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E62" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>其它</t>
+        </is>
+      </c>
+      <c r="B63" s="27" t="inlineStr">
+        <is>
+          <t>恒顺陈醋（500ml/瓶）</t>
+        </is>
+      </c>
+      <c r="C63" s="28" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D63" s="29" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E63" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="30" t="inlineStr">
+        <is>
+          <t>其它</t>
+        </is>
+      </c>
+      <c r="B64" s="31" t="inlineStr">
+        <is>
+          <t>蜜蜂味精（454g/袋）</t>
+        </is>
+      </c>
+      <c r="C64" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D64" s="33" t="inlineStr">
+        <is>
+          <t>→ 0.00%</t>
+        </is>
+      </c>
+      <c r="E64" s="30" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="38" t="inlineStr">
+        <is>
+          <t>📊 共 56 个品种 | 上涨 3 | 下跌 4 | 持平 49 | 无对比 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="39" t="inlineStr">
+        <is>
+          <t>↑ 红色=涨  ↓ 绿色=跌  → 灰色=持平  — =无上日数据</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A66:E66"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -19469,10 +21116,10 @@
           <t>📂 蔬菜（32 个品种）</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n"/>
-      <c r="C4" s="19" t="n"/>
-      <c r="D4" s="19" t="n"/>
-      <c r="E4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
+      <c r="C4" s="20" t="n"/>
+      <c r="D4" s="20" t="n"/>
+      <c r="E4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -20280,10 +21927,10 @@
           <t>📂 水果（9 个品种）</t>
         </is>
       </c>
-      <c r="B37" s="19" t="n"/>
-      <c r="C37" s="19" t="n"/>
-      <c r="D37" s="19" t="n"/>
-      <c r="E37" s="19" t="n"/>
+      <c r="B37" s="20" t="n"/>
+      <c r="C37" s="20" t="n"/>
+      <c r="D37" s="20" t="n"/>
+      <c r="E37" s="21" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -20516,10 +22163,10 @@
           <t>📂 肉禽蛋（10 个品种）</t>
         </is>
       </c>
-      <c r="B47" s="19" t="n"/>
-      <c r="C47" s="19" t="n"/>
-      <c r="D47" s="19" t="n"/>
-      <c r="E47" s="19" t="n"/>
+      <c r="B47" s="20" t="n"/>
+      <c r="C47" s="20" t="n"/>
+      <c r="D47" s="20" t="n"/>
+      <c r="E47" s="21" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -20777,10 +22424,10 @@
           <t>📂 水产（6 个品种）</t>
         </is>
       </c>
-      <c r="B58" s="19" t="n"/>
-      <c r="C58" s="19" t="n"/>
-      <c r="D58" s="19" t="n"/>
-      <c r="E58" s="19" t="n"/>
+      <c r="B58" s="20" t="n"/>
+      <c r="C58" s="20" t="n"/>
+      <c r="D58" s="20" t="n"/>
+      <c r="E58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
@@ -20938,10 +22585,10 @@
           <t>📂 粮油（24 个品种）</t>
         </is>
       </c>
-      <c r="B65" s="19" t="n"/>
-      <c r="C65" s="19" t="n"/>
-      <c r="D65" s="19" t="n"/>
-      <c r="E65" s="19" t="n"/>
+      <c r="B65" s="20" t="n"/>
+      <c r="C65" s="20" t="n"/>
+      <c r="D65" s="20" t="n"/>
+      <c r="E65" s="21" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -21549,10 +23196,10 @@
           <t>📂 其它（7 个品种）</t>
         </is>
       </c>
-      <c r="B90" s="19" t="n"/>
-      <c r="C90" s="19" t="n"/>
-      <c r="D90" s="19" t="n"/>
-      <c r="E90" s="19" t="n"/>
+      <c r="B90" s="20" t="n"/>
+      <c r="C90" s="20" t="n"/>
+      <c r="D90" s="20" t="n"/>
+      <c r="E90" s="21" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">

</xml_diff>